<commit_message>
fix(funnel): Starlyn UI bug fixes from 06/10 QA round + $19.99 add-on
Fix 108 of 117 bugs from Starlyn-ALL_UI_Bug_Report_06102026.xlsx across
the 10 nebula/ funnels (3 partly fixed, 6 left for PM: legal entity,
palm reviews). Shared fixes: real Terms/Privacy links with 44px tap
targets, official-logo store badges, single clock icon on time inputs,
chevrons on date selects, "Due today" shows the price only, opaque
sticky paywall bars, a CTA in the first view at 375x667, header-height
offset on loader/result screens, step counters that follow the branch.
Bug sheet Status column updated.

Also carries the post-purchase $19.99 add-on report screen and brief
updates, and a null guard in qa_capture.mjs for screens that re-render
while scrolling.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/funnel/funnel-testing/nebula/Starlyn-ALL_UI_Bug_Report_06102026.xlsx
+++ b/funnel/funnel-testing/nebula/Starlyn-ALL_UI_Bug_Report_06102026.xlsx
@@ -1307,7 +1307,7 @@
       </c>
       <c r="J2" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -1357,7 +1357,7 @@
       </c>
       <c r="J3" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Partly fixed</t>
         </is>
       </c>
     </row>
@@ -1407,7 +1407,7 @@
       </c>
       <c r="J4" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -1457,7 +1457,7 @@
       </c>
       <c r="J5" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -1507,7 +1507,7 @@
       </c>
       <c r="J6" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -1557,7 +1557,7 @@
       </c>
       <c r="J7" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -1607,7 +1607,7 @@
       </c>
       <c r="J8" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -1657,7 +1657,7 @@
       </c>
       <c r="J9" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -1707,7 +1707,7 @@
       </c>
       <c r="J10" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -1757,7 +1757,7 @@
       </c>
       <c r="J11" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -1807,7 +1807,7 @@
       </c>
       <c r="J12" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -1857,7 +1857,7 @@
       </c>
       <c r="J13" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -1907,7 +1907,7 @@
       </c>
       <c r="J14" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -1957,7 +1957,7 @@
       </c>
       <c r="J15" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -2007,7 +2007,7 @@
       </c>
       <c r="J16" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -2057,7 +2057,7 @@
       </c>
       <c r="J17" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -2107,7 +2107,7 @@
       </c>
       <c r="J18" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -2157,7 +2157,7 @@
       </c>
       <c r="J19" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -2207,7 +2207,7 @@
       </c>
       <c r="J20" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -2257,7 +2257,7 @@
       </c>
       <c r="J21" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -2307,7 +2307,7 @@
       </c>
       <c r="J22" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -2357,7 +2357,7 @@
       </c>
       <c r="J23" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -2407,7 +2407,7 @@
       </c>
       <c r="J24" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -2457,7 +2457,7 @@
       </c>
       <c r="J25" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -2507,7 +2507,7 @@
       </c>
       <c r="J26" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -2557,7 +2557,7 @@
       </c>
       <c r="J27" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -2607,7 +2607,7 @@
       </c>
       <c r="J28" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Cần PM</t>
         </is>
       </c>
     </row>
@@ -2657,7 +2657,7 @@
       </c>
       <c r="J29" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -2707,7 +2707,7 @@
       </c>
       <c r="J30" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -2757,7 +2757,7 @@
       </c>
       <c r="J31" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -2807,7 +2807,7 @@
       </c>
       <c r="J32" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -2857,7 +2857,7 @@
       </c>
       <c r="J33" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -2907,7 +2907,7 @@
       </c>
       <c r="J34" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -2957,7 +2957,7 @@
       </c>
       <c r="J35" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -3007,7 +3007,7 @@
       </c>
       <c r="J36" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -3057,7 +3057,7 @@
       </c>
       <c r="J37" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Cần PM</t>
         </is>
       </c>
     </row>
@@ -3107,7 +3107,7 @@
       </c>
       <c r="J38" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -3157,7 +3157,7 @@
       </c>
       <c r="J39" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -3207,7 +3207,7 @@
       </c>
       <c r="J40" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -3257,7 +3257,7 @@
       </c>
       <c r="J41" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Partly fixed</t>
         </is>
       </c>
     </row>
@@ -3307,7 +3307,7 @@
       </c>
       <c r="J42" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -3357,7 +3357,7 @@
       </c>
       <c r="J43" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -3407,7 +3407,7 @@
       </c>
       <c r="J44" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -3457,7 +3457,7 @@
       </c>
       <c r="J45" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -3507,7 +3507,7 @@
       </c>
       <c r="J46" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -3557,7 +3557,7 @@
       </c>
       <c r="J47" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -3607,7 +3607,7 @@
       </c>
       <c r="J48" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Cần PM</t>
         </is>
       </c>
     </row>
@@ -3657,7 +3657,7 @@
       </c>
       <c r="J49" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -3707,7 +3707,7 @@
       </c>
       <c r="J50" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -3757,7 +3757,7 @@
       </c>
       <c r="J51" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -3807,7 +3807,7 @@
       </c>
       <c r="J52" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -3857,7 +3857,7 @@
       </c>
       <c r="J53" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -3907,7 +3907,7 @@
       </c>
       <c r="J54" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -3957,7 +3957,7 @@
       </c>
       <c r="J55" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -4007,7 +4007,7 @@
       </c>
       <c r="J56" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -4057,7 +4057,7 @@
       </c>
       <c r="J57" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -4107,7 +4107,7 @@
       </c>
       <c r="J58" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -4157,7 +4157,7 @@
       </c>
       <c r="J59" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Partly fixed</t>
         </is>
       </c>
     </row>
@@ -4207,7 +4207,7 @@
       </c>
       <c r="J60" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -4257,7 +4257,7 @@
       </c>
       <c r="J61" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -4307,7 +4307,7 @@
       </c>
       <c r="J62" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -4357,7 +4357,7 @@
       </c>
       <c r="J63" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -4407,7 +4407,7 @@
       </c>
       <c r="J64" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -4457,7 +4457,7 @@
       </c>
       <c r="J65" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -4507,7 +4507,7 @@
       </c>
       <c r="J66" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -4557,7 +4557,7 @@
       </c>
       <c r="J67" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -4607,7 +4607,7 @@
       </c>
       <c r="J68" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -4657,7 +4657,7 @@
       </c>
       <c r="J69" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Cần PM</t>
         </is>
       </c>
     </row>
@@ -4707,7 +4707,7 @@
       </c>
       <c r="J70" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -4757,7 +4757,7 @@
       </c>
       <c r="J71" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -4807,7 +4807,7 @@
       </c>
       <c r="J72" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -4857,7 +4857,7 @@
       </c>
       <c r="J73" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -4907,7 +4907,7 @@
       </c>
       <c r="J74" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -4957,7 +4957,7 @@
       </c>
       <c r="J75" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -5007,7 +5007,7 @@
       </c>
       <c r="J76" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -5057,7 +5057,7 @@
       </c>
       <c r="J77" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -5107,7 +5107,7 @@
       </c>
       <c r="J78" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -5157,7 +5157,7 @@
       </c>
       <c r="J79" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -5207,7 +5207,7 @@
       </c>
       <c r="J80" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -5257,7 +5257,7 @@
       </c>
       <c r="J81" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -5307,7 +5307,7 @@
       </c>
       <c r="J82" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -5357,7 +5357,7 @@
       </c>
       <c r="J83" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Cần PM</t>
         </is>
       </c>
     </row>
@@ -5407,7 +5407,7 @@
       </c>
       <c r="J84" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -5457,7 +5457,7 @@
       </c>
       <c r="J85" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -5507,7 +5507,7 @@
       </c>
       <c r="J86" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -5557,7 +5557,7 @@
       </c>
       <c r="J87" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -5607,7 +5607,7 @@
       </c>
       <c r="J88" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -5657,7 +5657,7 @@
       </c>
       <c r="J89" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -5707,7 +5707,7 @@
       </c>
       <c r="J90" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -5757,7 +5757,7 @@
       </c>
       <c r="J91" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -5807,7 +5807,7 @@
       </c>
       <c r="J92" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -5857,7 +5857,7 @@
       </c>
       <c r="J93" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -5907,7 +5907,7 @@
       </c>
       <c r="J94" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -5957,7 +5957,7 @@
       </c>
       <c r="J95" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -6007,7 +6007,7 @@
       </c>
       <c r="J96" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -6057,7 +6057,7 @@
       </c>
       <c r="J97" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -6107,7 +6107,7 @@
       </c>
       <c r="J98" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -6157,7 +6157,7 @@
       </c>
       <c r="J99" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -6207,7 +6207,7 @@
       </c>
       <c r="J100" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -6257,7 +6257,7 @@
       </c>
       <c r="J101" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -6307,7 +6307,7 @@
       </c>
       <c r="J102" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -6357,7 +6357,7 @@
       </c>
       <c r="J103" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -6407,7 +6407,7 @@
       </c>
       <c r="J104" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -6457,7 +6457,7 @@
       </c>
       <c r="J105" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -6507,7 +6507,7 @@
       </c>
       <c r="J106" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -6557,7 +6557,7 @@
       </c>
       <c r="J107" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -6607,7 +6607,7 @@
       </c>
       <c r="J108" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -6657,7 +6657,7 @@
       </c>
       <c r="J109" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -6707,7 +6707,7 @@
       </c>
       <c r="J110" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -6757,7 +6757,7 @@
       </c>
       <c r="J111" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -6807,7 +6807,7 @@
       </c>
       <c r="J112" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -6857,7 +6857,7 @@
       </c>
       <c r="J113" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -6907,7 +6907,7 @@
       </c>
       <c r="J114" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -6957,7 +6957,7 @@
       </c>
       <c r="J115" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -7007,7 +7007,7 @@
       </c>
       <c r="J116" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -7057,7 +7057,7 @@
       </c>
       <c r="J117" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Cần PM</t>
         </is>
       </c>
     </row>
@@ -7107,7 +7107,7 @@
       </c>
       <c r="J118" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>

</xml_diff>